<commit_message>
test: troca dados pessoais reais por fictícios nos testes e fixtures (LGPD)
O repositório é público e os testes traziam dados de pessoas reais: um
funcionário (nome, CPF, PIS, nascimento, CTPS, salário) nas fixtures do IOB
SAGE e a planilha de apontamento de um cliente com 19 nomes.

- Valores fictícios do mesmo tamanho; nos backups custom o bloco zlib foi
  refeito com o mesmo tamanho (TOC e posições intactos).
- Planilha com "FUNCIONARIO FICTICIO NN" e teste que barra outro nome.
- O histórico do Git ainda tem os dados antigos (decisão do Paulo).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VnUByyvYyNGjaYJrpNadak
</commit_message>
<xml_diff>
--- a/services/folha/__tests__/fixtures/FASTWELD_-_0109.xlsx
+++ b/services/folha/__tests__/fixtures/FASTWELD_-_0109.xlsx
@@ -63,7 +63,7 @@
     <t>000109</t>
   </si>
   <si>
-    <t>ALEXANDRE ARAUJO DOS SANTOS</t>
+    <t>FUNCIONARIO FICTICIO 01</t>
   </si>
   <si>
     <t>FALTAS (DIAS)</t>
@@ -99,13 +99,13 @@
     <t>000107</t>
   </si>
   <si>
-    <t>ANTONIO SOUZA EVARISTO</t>
+    <t>FUNCIONARIO FICTICIO 02</t>
   </si>
   <si>
     <t>000019</t>
   </si>
   <si>
-    <t>ARNEZILDO REINALDO DE SOUSA</t>
+    <t>FUNCIONARIO FICTICIO 03</t>
   </si>
   <si>
     <t>0001</t>
@@ -117,13 +117,13 @@
     <t>000137</t>
   </si>
   <si>
-    <t>CARLOS ALBERTO DA SILVA</t>
+    <t>FUNCIONARIO FICTICIO 04</t>
   </si>
   <si>
     <t>000125</t>
   </si>
   <si>
-    <t>CARLOS RODRIGUES VIANA DOS SANTO</t>
+    <t>FUNCIONARIO FICTICIO 05</t>
   </si>
   <si>
     <t>CONTRIBUIÇÃO ASSISTENCIAL</t>
@@ -132,79 +132,79 @@
     <t>000152</t>
   </si>
   <si>
-    <t>EDUARDO ALVES AMBROSIO</t>
+    <t>FUNCIONARIO FICTICIO 06</t>
   </si>
   <si>
     <t>000120</t>
   </si>
   <si>
-    <t>ELOETE CRISTIANE RAMOS CARDOSO</t>
+    <t>FUNCIONARIO FICTICIO 07</t>
   </si>
   <si>
     <t>000148</t>
   </si>
   <si>
-    <t>JOHNATA ADRIANO DA SILVA</t>
+    <t>FUNCIONARIO FICTICIO 08</t>
   </si>
   <si>
     <t>000142</t>
   </si>
   <si>
-    <t>JOSE FELIPE DE ARRUDA SILVA</t>
+    <t>FUNCIONARIO FICTICIO 09</t>
   </si>
   <si>
     <t>000016</t>
   </si>
   <si>
-    <t>JOSE LUIZ DOS SANTOS SAMPAIO</t>
+    <t>FUNCIONARIO FICTICIO 10</t>
   </si>
   <si>
     <t>000055</t>
   </si>
   <si>
-    <t>JOSI SANTOS DE AZEVEDO FINARDI</t>
+    <t>FUNCIONARIO FICTICIO 11</t>
   </si>
   <si>
     <t>000138</t>
   </si>
   <si>
-    <t>LANA XAVIER DE MOURA</t>
+    <t>FUNCIONARIO FICTICIO 12</t>
   </si>
   <si>
     <t>000086</t>
   </si>
   <si>
-    <t>LEANDRO HELENO COSTA DE ALBUQUE</t>
+    <t>FUNCIONARIO FICTICIO 13</t>
   </si>
   <si>
     <t>000136</t>
   </si>
   <si>
-    <t>MARIA JOSE GOMES DE OLIVEIRA</t>
+    <t>FUNCIONARIO FICTICIO 14</t>
   </si>
   <si>
     <t>000112</t>
   </si>
   <si>
-    <t>MASTERSON DE MATOS</t>
+    <t>FUNCIONARIO FICTICIO 15</t>
   </si>
   <si>
     <t>000154</t>
   </si>
   <si>
-    <t>PAULO FERNANDES BALAN</t>
+    <t>FUNCIONARIO FICTICIO 16</t>
   </si>
   <si>
     <t>000098</t>
   </si>
   <si>
-    <t>SONIA CRISTINA SILVA</t>
+    <t>FUNCIONARIO FICTICIO 17</t>
   </si>
   <si>
     <t>000132</t>
   </si>
   <si>
-    <t>VANDERLANDO CONCEIÇÃO SILVA</t>
+    <t>FUNCIONARIO FICTICIO 18</t>
   </si>
   <si>
     <t>PENSÃO ALIMENTÍCIA</t>
@@ -213,7 +213,7 @@
     <t>000036</t>
   </si>
   <si>
-    <t>VINICIUS MEDEIROS BOTELHO</t>
+    <t>FUNCIONARIO FICTICIO 19</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
test: troca dados pessoais reais por fictícios nos testes e fixtures (LGPD) (#238)
O repositório é público e os testes traziam dados de pessoas reais: um
funcionário (nome, CPF, PIS, nascimento, CTPS, salário) nas fixtures do IOB
SAGE e a planilha de apontamento de um cliente com 19 nomes.

- Valores fictícios do mesmo tamanho; nos backups custom o bloco zlib foi
  refeito com o mesmo tamanho (TOC e posições intactos).
- Planilha com "FUNCIONARIO FICTICIO NN" e teste que barra outro nome.
- O histórico do Git ainda tem os dados antigos (decisão do Paulo).


Claude-Session: https://claude.ai/code/session_01VnUByyvYyNGjaYJrpNadak

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/services/folha/__tests__/fixtures/FASTWELD_-_0109.xlsx
+++ b/services/folha/__tests__/fixtures/FASTWELD_-_0109.xlsx
@@ -63,7 +63,7 @@
     <t>000109</t>
   </si>
   <si>
-    <t>ALEXANDRE ARAUJO DOS SANTOS</t>
+    <t>FUNCIONARIO FICTICIO 01</t>
   </si>
   <si>
     <t>FALTAS (DIAS)</t>
@@ -99,13 +99,13 @@
     <t>000107</t>
   </si>
   <si>
-    <t>ANTONIO SOUZA EVARISTO</t>
+    <t>FUNCIONARIO FICTICIO 02</t>
   </si>
   <si>
     <t>000019</t>
   </si>
   <si>
-    <t>ARNEZILDO REINALDO DE SOUSA</t>
+    <t>FUNCIONARIO FICTICIO 03</t>
   </si>
   <si>
     <t>0001</t>
@@ -117,13 +117,13 @@
     <t>000137</t>
   </si>
   <si>
-    <t>CARLOS ALBERTO DA SILVA</t>
+    <t>FUNCIONARIO FICTICIO 04</t>
   </si>
   <si>
     <t>000125</t>
   </si>
   <si>
-    <t>CARLOS RODRIGUES VIANA DOS SANTO</t>
+    <t>FUNCIONARIO FICTICIO 05</t>
   </si>
   <si>
     <t>CONTRIBUIÇÃO ASSISTENCIAL</t>
@@ -132,79 +132,79 @@
     <t>000152</t>
   </si>
   <si>
-    <t>EDUARDO ALVES AMBROSIO</t>
+    <t>FUNCIONARIO FICTICIO 06</t>
   </si>
   <si>
     <t>000120</t>
   </si>
   <si>
-    <t>ELOETE CRISTIANE RAMOS CARDOSO</t>
+    <t>FUNCIONARIO FICTICIO 07</t>
   </si>
   <si>
     <t>000148</t>
   </si>
   <si>
-    <t>JOHNATA ADRIANO DA SILVA</t>
+    <t>FUNCIONARIO FICTICIO 08</t>
   </si>
   <si>
     <t>000142</t>
   </si>
   <si>
-    <t>JOSE FELIPE DE ARRUDA SILVA</t>
+    <t>FUNCIONARIO FICTICIO 09</t>
   </si>
   <si>
     <t>000016</t>
   </si>
   <si>
-    <t>JOSE LUIZ DOS SANTOS SAMPAIO</t>
+    <t>FUNCIONARIO FICTICIO 10</t>
   </si>
   <si>
     <t>000055</t>
   </si>
   <si>
-    <t>JOSI SANTOS DE AZEVEDO FINARDI</t>
+    <t>FUNCIONARIO FICTICIO 11</t>
   </si>
   <si>
     <t>000138</t>
   </si>
   <si>
-    <t>LANA XAVIER DE MOURA</t>
+    <t>FUNCIONARIO FICTICIO 12</t>
   </si>
   <si>
     <t>000086</t>
   </si>
   <si>
-    <t>LEANDRO HELENO COSTA DE ALBUQUE</t>
+    <t>FUNCIONARIO FICTICIO 13</t>
   </si>
   <si>
     <t>000136</t>
   </si>
   <si>
-    <t>MARIA JOSE GOMES DE OLIVEIRA</t>
+    <t>FUNCIONARIO FICTICIO 14</t>
   </si>
   <si>
     <t>000112</t>
   </si>
   <si>
-    <t>MASTERSON DE MATOS</t>
+    <t>FUNCIONARIO FICTICIO 15</t>
   </si>
   <si>
     <t>000154</t>
   </si>
   <si>
-    <t>PAULO FERNANDES BALAN</t>
+    <t>FUNCIONARIO FICTICIO 16</t>
   </si>
   <si>
     <t>000098</t>
   </si>
   <si>
-    <t>SONIA CRISTINA SILVA</t>
+    <t>FUNCIONARIO FICTICIO 17</t>
   </si>
   <si>
     <t>000132</t>
   </si>
   <si>
-    <t>VANDERLANDO CONCEIÇÃO SILVA</t>
+    <t>FUNCIONARIO FICTICIO 18</t>
   </si>
   <si>
     <t>PENSÃO ALIMENTÍCIA</t>
@@ -213,7 +213,7 @@
     <t>000036</t>
   </si>
   <si>
-    <t>VINICIUS MEDEIROS BOTELHO</t>
+    <t>FUNCIONARIO FICTICIO 19</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Revert "test: troca dados pessoais reais por fictícios nos testes e fixtures (LGPD) (#238)"
A pedido do Paulo: os arquivos de teste e as fixtures voltam a ser
exatamente como estavam antes do #238. O #238 não tinha alterado dados
do sistema, só cópias usadas pelos testes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VnUByyvYyNGjaYJrpNadak
</commit_message>
<xml_diff>
--- a/services/folha/__tests__/fixtures/FASTWELD_-_0109.xlsx
+++ b/services/folha/__tests__/fixtures/FASTWELD_-_0109.xlsx
@@ -63,7 +63,7 @@
     <t>000109</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 01</t>
+    <t>ALEXANDRE ARAUJO DOS SANTOS</t>
   </si>
   <si>
     <t>FALTAS (DIAS)</t>
@@ -99,13 +99,13 @@
     <t>000107</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 02</t>
+    <t>ANTONIO SOUZA EVARISTO</t>
   </si>
   <si>
     <t>000019</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 03</t>
+    <t>ARNEZILDO REINALDO DE SOUSA</t>
   </si>
   <si>
     <t>0001</t>
@@ -117,13 +117,13 @@
     <t>000137</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 04</t>
+    <t>CARLOS ALBERTO DA SILVA</t>
   </si>
   <si>
     <t>000125</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 05</t>
+    <t>CARLOS RODRIGUES VIANA DOS SANTO</t>
   </si>
   <si>
     <t>CONTRIBUIÇÃO ASSISTENCIAL</t>
@@ -132,79 +132,79 @@
     <t>000152</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 06</t>
+    <t>EDUARDO ALVES AMBROSIO</t>
   </si>
   <si>
     <t>000120</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 07</t>
+    <t>ELOETE CRISTIANE RAMOS CARDOSO</t>
   </si>
   <si>
     <t>000148</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 08</t>
+    <t>JOHNATA ADRIANO DA SILVA</t>
   </si>
   <si>
     <t>000142</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 09</t>
+    <t>JOSE FELIPE DE ARRUDA SILVA</t>
   </si>
   <si>
     <t>000016</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 10</t>
+    <t>JOSE LUIZ DOS SANTOS SAMPAIO</t>
   </si>
   <si>
     <t>000055</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 11</t>
+    <t>JOSI SANTOS DE AZEVEDO FINARDI</t>
   </si>
   <si>
     <t>000138</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 12</t>
+    <t>LANA XAVIER DE MOURA</t>
   </si>
   <si>
     <t>000086</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 13</t>
+    <t>LEANDRO HELENO COSTA DE ALBUQUE</t>
   </si>
   <si>
     <t>000136</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 14</t>
+    <t>MARIA JOSE GOMES DE OLIVEIRA</t>
   </si>
   <si>
     <t>000112</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 15</t>
+    <t>MASTERSON DE MATOS</t>
   </si>
   <si>
     <t>000154</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 16</t>
+    <t>PAULO FERNANDES BALAN</t>
   </si>
   <si>
     <t>000098</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 17</t>
+    <t>SONIA CRISTINA SILVA</t>
   </si>
   <si>
     <t>000132</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 18</t>
+    <t>VANDERLANDO CONCEIÇÃO SILVA</t>
   </si>
   <si>
     <t>PENSÃO ALIMENTÍCIA</t>
@@ -213,7 +213,7 @@
     <t>000036</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 19</t>
+    <t>VINICIUS MEDEIROS BOTELHO</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Revert "test: troca dados pessoais reais por fictícios nos testes e fixtures (LGPD) (#238)" (#239)
A pedido do Paulo: os arquivos de teste e as fixtures voltam a ser
exatamente como estavam antes do #238. O #238 não tinha alterado dados
do sistema, só cópias usadas pelos testes.


Claude-Session: https://claude.ai/code/session_01VnUByyvYyNGjaYJrpNadak

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/services/folha/__tests__/fixtures/FASTWELD_-_0109.xlsx
+++ b/services/folha/__tests__/fixtures/FASTWELD_-_0109.xlsx
@@ -63,7 +63,7 @@
     <t>000109</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 01</t>
+    <t>ALEXANDRE ARAUJO DOS SANTOS</t>
   </si>
   <si>
     <t>FALTAS (DIAS)</t>
@@ -99,13 +99,13 @@
     <t>000107</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 02</t>
+    <t>ANTONIO SOUZA EVARISTO</t>
   </si>
   <si>
     <t>000019</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 03</t>
+    <t>ARNEZILDO REINALDO DE SOUSA</t>
   </si>
   <si>
     <t>0001</t>
@@ -117,13 +117,13 @@
     <t>000137</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 04</t>
+    <t>CARLOS ALBERTO DA SILVA</t>
   </si>
   <si>
     <t>000125</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 05</t>
+    <t>CARLOS RODRIGUES VIANA DOS SANTO</t>
   </si>
   <si>
     <t>CONTRIBUIÇÃO ASSISTENCIAL</t>
@@ -132,79 +132,79 @@
     <t>000152</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 06</t>
+    <t>EDUARDO ALVES AMBROSIO</t>
   </si>
   <si>
     <t>000120</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 07</t>
+    <t>ELOETE CRISTIANE RAMOS CARDOSO</t>
   </si>
   <si>
     <t>000148</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 08</t>
+    <t>JOHNATA ADRIANO DA SILVA</t>
   </si>
   <si>
     <t>000142</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 09</t>
+    <t>JOSE FELIPE DE ARRUDA SILVA</t>
   </si>
   <si>
     <t>000016</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 10</t>
+    <t>JOSE LUIZ DOS SANTOS SAMPAIO</t>
   </si>
   <si>
     <t>000055</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 11</t>
+    <t>JOSI SANTOS DE AZEVEDO FINARDI</t>
   </si>
   <si>
     <t>000138</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 12</t>
+    <t>LANA XAVIER DE MOURA</t>
   </si>
   <si>
     <t>000086</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 13</t>
+    <t>LEANDRO HELENO COSTA DE ALBUQUE</t>
   </si>
   <si>
     <t>000136</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 14</t>
+    <t>MARIA JOSE GOMES DE OLIVEIRA</t>
   </si>
   <si>
     <t>000112</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 15</t>
+    <t>MASTERSON DE MATOS</t>
   </si>
   <si>
     <t>000154</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 16</t>
+    <t>PAULO FERNANDES BALAN</t>
   </si>
   <si>
     <t>000098</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 17</t>
+    <t>SONIA CRISTINA SILVA</t>
   </si>
   <si>
     <t>000132</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 18</t>
+    <t>VANDERLANDO CONCEIÇÃO SILVA</t>
   </si>
   <si>
     <t>PENSÃO ALIMENTÍCIA</t>
@@ -213,7 +213,7 @@
     <t>000036</t>
   </si>
   <si>
-    <t>FUNCIONARIO FICTICIO 19</t>
+    <t>VINICIUS MEDEIROS BOTELHO</t>
   </si>
 </sst>
 </file>

</xml_diff>